<commit_message>
update dictionary and configs
</commit_message>
<xml_diff>
--- a/data_preparation/docs/data_dictionary.xlsx
+++ b/data_preparation/docs/data_dictionary.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\aleks\hackathon\Artraid\data_preparation\docs\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\aleks\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{679CF33D-8A98-475E-800A-E52528216B6A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2EA326F2-5111-4841-B308-04EF6814A585}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -16,7 +16,7 @@
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$A$1:$I$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$A$1:$J$1</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="128" uniqueCount="84">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="205" uniqueCount="119">
   <si>
     <t>Столбец</t>
   </si>
@@ -288,6 +288,111 @@
   </si>
   <si>
     <t>если в сумме несколько товаров отображается стоимость +G7+H2:H36+H2:H38+G7+H2:H+H2:H15</t>
+  </si>
+  <si>
+    <t>update 07/04</t>
+  </si>
+  <si>
+    <t>lead_source_category - используем этот фичу</t>
+  </si>
+  <si>
+    <t>has_promo, lead_source_category, is_yur</t>
+  </si>
+  <si>
+    <t>вытащить стоимость доставки, сделать флаг "бесплатная доставка"</t>
+  </si>
+  <si>
+    <t>has_yclid</t>
+  </si>
+  <si>
+    <t>bool</t>
+  </si>
+  <si>
+    <t>is_paid_mop</t>
+  </si>
+  <si>
+    <t>is_repeat_client</t>
+  </si>
+  <si>
+    <t>has_promo</t>
+  </si>
+  <si>
+    <t>lead_source_category</t>
+  </si>
+  <si>
+    <t>is_yur</t>
+  </si>
+  <si>
+    <t>n_product_categories</t>
+  </si>
+  <si>
+    <t>has_маска</t>
+  </si>
+  <si>
+    <t>has_наколенник</t>
+  </si>
+  <si>
+    <t>has_бандаж_шейный</t>
+  </si>
+  <si>
+    <t>has_повязка</t>
+  </si>
+  <si>
+    <t>has_напульсник</t>
+  </si>
+  <si>
+    <t>has_обувь</t>
+  </si>
+  <si>
+    <t>has_подушка</t>
+  </si>
+  <si>
+    <t>has_матрас</t>
+  </si>
+  <si>
+    <t>has_пояс</t>
+  </si>
+  <si>
+    <t>has_аксессуары</t>
+  </si>
+  <si>
+    <t>has_крем</t>
+  </si>
+  <si>
+    <t>Целевой тип</t>
+  </si>
+  <si>
+    <t>datetime64[s]</t>
+  </si>
+  <si>
+    <t>category</t>
+  </si>
+  <si>
+    <t>Int64</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> category</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> str</t>
+  </si>
+  <si>
+    <t>datetime64[us]</t>
+  </si>
+  <si>
+    <t>price_group</t>
+  </si>
+  <si>
+    <t>delivery_group</t>
+  </si>
+  <si>
+    <t>region</t>
+  </si>
+  <si>
+    <t>shipping_cost</t>
+  </si>
+  <si>
+    <t>category?</t>
   </si>
 </sst>
 </file>
@@ -350,7 +455,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="4">
+  <borders count="5">
     <border>
       <left/>
       <right/>
@@ -389,18 +494,26 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="20">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
@@ -408,16 +521,10 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="4" xfId="0" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -720,1120 +827,1576 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:J68"/>
+  <dimension ref="A1:K68"/>
   <sheetFormatPr defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="34" style="5" customWidth="1"/>
-    <col min="2" max="2" width="18.88671875" style="5" customWidth="1"/>
-    <col min="3" max="3" width="22.33203125" style="5" customWidth="1"/>
-    <col min="4" max="7" width="18.88671875" style="5" customWidth="1"/>
-    <col min="8" max="8" width="37.33203125" style="5" customWidth="1"/>
-    <col min="9" max="9" width="40" style="5" customWidth="1"/>
-    <col min="10" max="10" width="54.6640625" style="6" customWidth="1"/>
-    <col min="11" max="11" width="17.88671875" style="5" customWidth="1"/>
-    <col min="12" max="16384" width="8.88671875" style="5"/>
+    <col min="1" max="1" width="34" customWidth="1"/>
+    <col min="2" max="2" width="18.88671875" customWidth="1"/>
+    <col min="3" max="3" width="22" customWidth="1"/>
+    <col min="4" max="4" width="22.33203125" customWidth="1"/>
+    <col min="5" max="8" width="18.88671875" customWidth="1"/>
+    <col min="9" max="9" width="37.33203125" customWidth="1"/>
+    <col min="10" max="10" width="40" style="5" customWidth="1"/>
+    <col min="11" max="11" width="54.6640625" style="5" customWidth="1"/>
+    <col min="12" max="12" width="17.88671875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="7" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="8" t="s">
+    <row r="1" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A1" s="6" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="7" t="s">
         <v>48</v>
       </c>
-      <c r="C1" s="8" t="s">
+      <c r="C1" s="7" t="s">
+        <v>107</v>
+      </c>
+      <c r="D1" s="7" t="s">
         <v>1</v>
       </c>
-      <c r="D1" s="8" t="s">
+      <c r="E1" s="7" t="s">
         <v>2</v>
       </c>
-      <c r="E1" s="8" t="s">
+      <c r="F1" s="7" t="s">
         <v>3</v>
       </c>
-      <c r="F1" s="9" t="s">
+      <c r="G1" s="8" t="s">
         <v>4</v>
       </c>
-      <c r="G1" s="8" t="s">
+      <c r="H1" s="7" t="s">
         <v>42</v>
       </c>
-      <c r="H1" s="10" t="s">
+      <c r="I1" s="9" t="s">
         <v>49</v>
       </c>
-      <c r="I1" s="10" t="s">
+      <c r="J1" s="11" t="s">
         <v>50</v>
       </c>
-    </row>
-    <row r="2" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="K1" s="11" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="2" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
         <v>51</v>
       </c>
       <c r="B2" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="C2" s="1">
+      <c r="C2" s="1"/>
+      <c r="D2" s="1">
         <v>18808</v>
       </c>
-      <c r="D2" s="1">
+      <c r="E2" s="1">
         <v>99.58</v>
       </c>
-      <c r="E2" s="1">
+      <c r="F2" s="1">
         <v>79</v>
       </c>
-      <c r="F2" s="1">
+      <c r="G2" s="1">
         <v>17</v>
       </c>
-      <c r="G2" s="1"/>
-      <c r="H2" s="18" t="s">
+      <c r="H2" s="1"/>
+      <c r="I2" t="s">
         <v>52</v>
       </c>
-      <c r="I2" s="18" t="s">
+      <c r="J2" s="5" t="s">
         <v>83</v>
       </c>
     </row>
-    <row r="3" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="1" t="s">
         <v>53</v>
       </c>
       <c r="B3" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="C3" s="1">
+      <c r="C3" s="1"/>
+      <c r="D3" s="1">
         <v>18436</v>
       </c>
-      <c r="D3" s="1">
+      <c r="E3" s="1">
         <v>97.61</v>
       </c>
-      <c r="E3" s="1">
+      <c r="F3" s="1">
         <v>451</v>
       </c>
-      <c r="F3" s="1">
+      <c r="G3" s="1">
         <v>1</v>
       </c>
-      <c r="G3" s="1"/>
-      <c r="H3" s="18" t="s">
+      <c r="H3" s="1"/>
+      <c r="I3" t="s">
         <v>54</v>
       </c>
-      <c r="I3" s="18" t="s">
+      <c r="J3" s="5" t="s">
         <v>55</v>
       </c>
     </row>
-    <row r="4" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="1" t="s">
         <v>56</v>
       </c>
       <c r="B4" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="C4" s="1">
+      <c r="C4" s="1"/>
+      <c r="D4" s="1">
         <v>18086</v>
       </c>
-      <c r="D4" s="1">
+      <c r="E4" s="1">
         <v>95.76</v>
       </c>
-      <c r="E4" s="1">
+      <c r="F4" s="1">
         <v>801</v>
       </c>
-      <c r="F4" s="1">
+      <c r="G4" s="1">
         <v>1</v>
       </c>
-      <c r="G4" s="1"/>
-      <c r="H4" s="18"/>
-      <c r="I4" s="18" t="s">
+      <c r="H4" s="1"/>
+      <c r="J4" s="5" t="s">
         <v>57</v>
       </c>
     </row>
-    <row r="5" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="1" t="s">
         <v>58</v>
       </c>
       <c r="B5" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="C5" s="1">
+      <c r="C5" s="1"/>
+      <c r="D5" s="1">
         <v>18064</v>
       </c>
-      <c r="D5" s="1">
+      <c r="E5" s="1">
         <v>95.64</v>
       </c>
-      <c r="E5" s="1">
+      <c r="F5" s="1">
         <v>823</v>
       </c>
-      <c r="F5" s="1">
+      <c r="G5" s="1">
         <v>1</v>
       </c>
-      <c r="G5" s="1"/>
-      <c r="H5" s="18"/>
-      <c r="I5" s="18" t="s">
+      <c r="H5" s="1"/>
+      <c r="J5" s="5" t="s">
         <v>57</v>
       </c>
     </row>
-    <row r="6" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="2" t="s">
         <v>17</v>
       </c>
       <c r="B6" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="C6" s="2">
+      <c r="C6" s="2" t="s">
+        <v>108</v>
+      </c>
+      <c r="D6" s="2">
         <v>16354</v>
       </c>
-      <c r="D6" s="2">
+      <c r="E6" s="2">
         <v>86.59</v>
-      </c>
-      <c r="E6" s="2">
-        <v>2533</v>
       </c>
       <c r="F6" s="2">
         <v>2533</v>
       </c>
-      <c r="G6" s="2"/>
-      <c r="H6" s="18"/>
-      <c r="I6" s="18"/>
-    </row>
-    <row r="7" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="G6" s="2">
+        <v>2533</v>
+      </c>
+      <c r="H6" s="2"/>
+    </row>
+    <row r="7" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="2" t="s">
         <v>16</v>
       </c>
       <c r="B7" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="C7" s="2">
+      <c r="C7" s="2" t="s">
+        <v>108</v>
+      </c>
+      <c r="D7" s="2">
         <v>16257</v>
       </c>
-      <c r="D7" s="2">
+      <c r="E7" s="2">
         <v>86.08</v>
-      </c>
-      <c r="E7" s="2">
-        <v>2630</v>
       </c>
       <c r="F7" s="2">
         <v>2630</v>
       </c>
-      <c r="G7" s="2"/>
-      <c r="H7" s="18" t="s">
+      <c r="G7" s="2">
+        <v>2630</v>
+      </c>
+      <c r="H7" s="2"/>
+      <c r="I7" t="s">
         <v>59</v>
       </c>
-      <c r="I7" s="18"/>
-    </row>
-    <row r="8" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    </row>
+    <row r="8" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" s="3" t="s">
         <v>32</v>
       </c>
       <c r="B8" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="C8" s="3">
+      <c r="C8" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="D8" s="3">
         <v>16118</v>
       </c>
-      <c r="D8" s="3">
+      <c r="E8" s="3">
         <v>85.34</v>
       </c>
-      <c r="E8" s="3">
+      <c r="F8" s="3">
         <v>2769</v>
       </c>
-      <c r="F8" s="3">
+      <c r="G8" s="3">
         <v>24</v>
       </c>
-      <c r="G8" s="3"/>
-      <c r="H8" s="18" t="s">
+      <c r="H8" s="3"/>
+      <c r="I8" t="s">
         <v>60</v>
       </c>
-      <c r="I8" s="18" t="s">
+      <c r="J8" s="5" t="s">
         <v>61</v>
       </c>
     </row>
-    <row r="9" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A9" s="2" t="s">
+    <row r="9" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A9" s="1" t="s">
         <v>40</v>
       </c>
-      <c r="B9" s="2" t="s">
-        <v>6</v>
-      </c>
-      <c r="C9" s="2">
+      <c r="B9" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="C9" s="1"/>
+      <c r="D9" s="1">
         <v>16026</v>
       </c>
-      <c r="D9" s="2">
+      <c r="E9" s="1">
         <v>84.85</v>
       </c>
-      <c r="E9" s="2">
+      <c r="F9" s="1">
         <v>2861</v>
       </c>
-      <c r="F9" s="2">
+      <c r="G9" s="1">
         <v>19</v>
       </c>
-      <c r="G9" s="2"/>
-      <c r="H9" s="18" t="s">
+      <c r="H9" s="1"/>
+      <c r="I9" t="s">
         <v>62</v>
       </c>
-      <c r="I9" s="18" t="s">
+      <c r="J9" s="5" t="s">
         <v>63</v>
       </c>
     </row>
-    <row r="10" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A10" s="1" t="s">
         <v>41</v>
       </c>
       <c r="B10" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="C10" s="1">
+      <c r="C10" s="1"/>
+      <c r="D10" s="1">
         <v>15825</v>
       </c>
-      <c r="D10" s="1">
+      <c r="E10" s="1">
         <v>83.79</v>
       </c>
-      <c r="E10" s="1">
+      <c r="F10" s="1">
         <v>3062</v>
       </c>
-      <c r="F10" s="1">
+      <c r="G10" s="1">
         <v>2799</v>
       </c>
-      <c r="G10" s="1"/>
-      <c r="H10" s="18" t="s">
+      <c r="H10" s="1"/>
+      <c r="I10" t="s">
         <v>47</v>
       </c>
-      <c r="I10" s="18" t="s">
+      <c r="J10" s="5" t="s">
         <v>64</v>
       </c>
     </row>
-    <row r="11" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A11" s="1" t="s">
         <v>65</v>
       </c>
       <c r="B11" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="C11" s="1">
+      <c r="C11" s="1"/>
+      <c r="D11" s="1">
         <v>15790</v>
       </c>
-      <c r="D11" s="1">
+      <c r="E11" s="1">
         <v>83.6</v>
       </c>
-      <c r="E11" s="1">
+      <c r="F11" s="1">
         <v>3097</v>
       </c>
-      <c r="F11" s="1">
+      <c r="G11" s="1">
         <v>1</v>
       </c>
-      <c r="G11" s="1"/>
-      <c r="H11" s="18"/>
-      <c r="I11" s="18" t="s">
+      <c r="H11" s="1"/>
+      <c r="J11" s="5" t="s">
         <v>57</v>
       </c>
     </row>
-    <row r="12" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A12" s="11" t="s">
+    <row r="12" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A12" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="B12" s="11" t="s">
-        <v>6</v>
-      </c>
-      <c r="C12" s="11">
+      <c r="B12" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="C12" s="1"/>
+      <c r="D12" s="1">
         <v>14255</v>
       </c>
-      <c r="D12" s="11">
+      <c r="E12" s="1">
         <v>75.48</v>
       </c>
-      <c r="E12" s="11">
+      <c r="F12" s="1">
         <v>4632</v>
       </c>
-      <c r="F12" s="11">
+      <c r="G12" s="1">
         <v>8</v>
       </c>
-      <c r="G12" s="11"/>
-      <c r="H12" s="18"/>
-      <c r="I12" s="18" t="s">
+      <c r="H12" s="1"/>
+      <c r="J12" s="5" t="s">
         <v>66</v>
       </c>
-    </row>
-    <row r="13" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="K12" s="5" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="13" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A13" s="1" t="s">
         <v>67</v>
       </c>
       <c r="B13" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="C13" s="1">
+      <c r="C13" s="1"/>
+      <c r="D13" s="1">
         <v>13770</v>
       </c>
-      <c r="D13" s="1">
+      <c r="E13" s="1">
         <v>72.91</v>
       </c>
-      <c r="E13" s="1">
+      <c r="F13" s="1">
         <v>5117</v>
       </c>
-      <c r="F13" s="1">
+      <c r="G13" s="1">
         <v>1</v>
       </c>
-      <c r="G13" s="1"/>
-      <c r="H13" s="18"/>
-      <c r="I13" s="18" t="s">
+      <c r="H13" s="1"/>
+      <c r="J13" s="5" t="s">
         <v>57</v>
       </c>
     </row>
-    <row r="14" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A14" s="3" t="s">
         <v>68</v>
       </c>
       <c r="B14" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="C14" s="3">
+      <c r="C14" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="D14" s="3">
         <v>11621</v>
       </c>
-      <c r="D14" s="3">
+      <c r="E14" s="3">
         <v>61.53</v>
       </c>
-      <c r="E14" s="3">
+      <c r="F14" s="3">
         <v>7266</v>
       </c>
-      <c r="F14" s="3">
+      <c r="G14" s="3">
         <v>1</v>
       </c>
-      <c r="G14" s="3"/>
-      <c r="H14" s="18"/>
-      <c r="I14" s="18"/>
-    </row>
-    <row r="15" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A15" s="2" t="s">
+      <c r="H14" s="3"/>
+    </row>
+    <row r="15" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A15" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="B15" s="2" t="s">
+      <c r="B15" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="C15" s="2">
+      <c r="C15" s="1"/>
+      <c r="D15" s="1">
         <v>10601</v>
       </c>
-      <c r="D15" s="2">
+      <c r="E15" s="1">
         <v>56.13</v>
       </c>
-      <c r="E15" s="2">
+      <c r="F15" s="1">
         <v>8286</v>
       </c>
-      <c r="F15" s="2">
+      <c r="G15" s="1">
         <v>182</v>
       </c>
-      <c r="G15" s="2"/>
-      <c r="H15" s="18" t="s">
+      <c r="H15" s="1"/>
+      <c r="I15" t="s">
         <v>44</v>
       </c>
-      <c r="I15" s="18" t="s">
+      <c r="J15" s="5" t="s">
         <v>69</v>
       </c>
     </row>
-    <row r="16" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A16" s="2" t="s">
         <v>33</v>
       </c>
       <c r="B16" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="C16" s="2">
+      <c r="C16" s="2" t="s">
+        <v>108</v>
+      </c>
+      <c r="D16" s="2">
         <v>9671</v>
       </c>
-      <c r="D16" s="2">
+      <c r="E16" s="2">
         <v>51.2</v>
       </c>
-      <c r="E16" s="2">
+      <c r="F16" s="2">
         <v>9216</v>
       </c>
-      <c r="F16" s="2">
+      <c r="G16" s="2">
         <v>179</v>
       </c>
-      <c r="G16" s="2"/>
-      <c r="H16" s="18"/>
-      <c r="I16" s="18"/>
-    </row>
-    <row r="17" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="H16" s="2"/>
+    </row>
+    <row r="17" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A17" s="1" t="s">
         <v>26</v>
       </c>
       <c r="B17" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="C17" s="1">
+      <c r="C17" s="1"/>
+      <c r="D17" s="1">
         <v>9048</v>
       </c>
-      <c r="D17" s="1">
+      <c r="E17" s="1">
         <v>47.91</v>
       </c>
-      <c r="E17" s="1">
+      <c r="F17" s="1">
         <v>9839</v>
       </c>
-      <c r="F17" s="1">
+      <c r="G17" s="1">
         <v>5</v>
       </c>
-      <c r="G17" s="1"/>
-      <c r="H17" s="18"/>
-      <c r="I17" s="18" t="s">
+      <c r="H17" s="1"/>
+      <c r="J17" s="5" t="s">
         <v>70</v>
       </c>
     </row>
-    <row r="18" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A18" s="11" t="s">
+    <row r="18" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A18" s="1" t="s">
         <v>71</v>
       </c>
-      <c r="B18" s="11" t="s">
-        <v>6</v>
-      </c>
-      <c r="C18" s="11">
+      <c r="B18" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="C18" s="1"/>
+      <c r="D18" s="1">
         <v>8971</v>
       </c>
-      <c r="D18" s="11">
+      <c r="E18" s="1">
         <v>47.5</v>
       </c>
-      <c r="E18" s="11">
+      <c r="F18" s="1">
         <v>9916</v>
       </c>
-      <c r="F18" s="11">
+      <c r="G18" s="1">
         <v>9907</v>
       </c>
-      <c r="G18" s="11"/>
-      <c r="H18" s="18"/>
-      <c r="I18" s="18" t="s">
+      <c r="H18" s="1"/>
+      <c r="J18" s="5" t="s">
         <v>72</v>
       </c>
     </row>
-    <row r="19" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A19" s="3" t="s">
         <v>34</v>
       </c>
       <c r="B19" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="C19" s="3">
+      <c r="C19" s="3" t="s">
+        <v>108</v>
+      </c>
+      <c r="D19" s="3">
         <v>7411</v>
       </c>
-      <c r="D19" s="3">
+      <c r="E19" s="3">
         <v>39.24</v>
       </c>
-      <c r="E19" s="3">
+      <c r="F19" s="3">
         <v>11476</v>
       </c>
-      <c r="F19" s="3">
+      <c r="G19" s="3">
         <v>261</v>
       </c>
-      <c r="G19" s="3"/>
-      <c r="H19" s="18" t="s">
+      <c r="H19" s="3"/>
+      <c r="I19" t="s">
         <v>46</v>
       </c>
-      <c r="I19" s="18" t="s">
+      <c r="J19" s="5" t="s">
         <v>73</v>
       </c>
     </row>
-    <row r="20" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A20" s="1" t="s">
         <v>37</v>
       </c>
       <c r="B20" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="C20" s="1">
+      <c r="C20" s="1"/>
+      <c r="D20" s="1">
         <v>7275</v>
       </c>
-      <c r="D20" s="1">
+      <c r="E20" s="1">
         <v>38.520000000000003</v>
       </c>
-      <c r="E20" s="1">
+      <c r="F20" s="1">
         <v>11612</v>
       </c>
-      <c r="F20" s="1">
+      <c r="G20" s="1">
         <v>1</v>
       </c>
-      <c r="G20" s="1"/>
-      <c r="H20" s="18"/>
-      <c r="I20" s="18" t="s">
+      <c r="H20" s="1"/>
+      <c r="J20" s="5" t="s">
         <v>57</v>
       </c>
     </row>
-    <row r="21" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A21" s="2" t="s">
         <v>25</v>
       </c>
       <c r="B21" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="C21" s="2">
+      <c r="C21" s="2" t="s">
+        <v>109</v>
+      </c>
+      <c r="D21" s="2">
         <v>6563</v>
       </c>
-      <c r="D21" s="2">
+      <c r="E21" s="2">
         <v>34.75</v>
       </c>
-      <c r="E21" s="2">
+      <c r="F21" s="2">
         <v>12324</v>
       </c>
-      <c r="F21" s="2">
-        <v>6</v>
-      </c>
-      <c r="G21" s="2"/>
-      <c r="H21" s="18"/>
-      <c r="I21" s="18" t="s">
+      <c r="G21" s="2">
+        <v>6</v>
+      </c>
+      <c r="H21" s="2"/>
+      <c r="J21" s="5" t="s">
         <v>74</v>
       </c>
     </row>
-    <row r="22" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A22" s="2" t="s">
         <v>38</v>
       </c>
       <c r="B22" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="C22" s="2">
+      <c r="C22" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="D22" s="2">
         <v>4926</v>
       </c>
-      <c r="D22" s="2">
+      <c r="E22" s="2">
         <v>26.08</v>
       </c>
-      <c r="E22" s="2">
+      <c r="F22" s="2">
         <v>13961</v>
       </c>
-      <c r="F22" s="2">
+      <c r="G22" s="2">
         <v>5709</v>
       </c>
-      <c r="G22" s="2"/>
-      <c r="H22" s="18"/>
-      <c r="I22" s="18"/>
-    </row>
-    <row r="23" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="H22" s="2"/>
+    </row>
+    <row r="23" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A23" s="2" t="s">
         <v>39</v>
       </c>
       <c r="B23" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="C23" s="2">
+      <c r="C23" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="D23" s="2">
         <v>4926</v>
       </c>
-      <c r="D23" s="2">
+      <c r="E23" s="2">
         <v>26.08</v>
       </c>
-      <c r="E23" s="2">
+      <c r="F23" s="2">
         <v>13961</v>
       </c>
-      <c r="F23" s="2">
+      <c r="G23" s="2">
         <v>19</v>
       </c>
-      <c r="G23" s="2"/>
-      <c r="H23" s="18" t="s">
+      <c r="H23" s="2"/>
+      <c r="I23" t="s">
         <v>45</v>
       </c>
-      <c r="I23" s="18" t="s">
+      <c r="J23" s="5" t="s">
         <v>75</v>
       </c>
     </row>
-    <row r="24" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A24" s="2" t="s">
         <v>15</v>
       </c>
       <c r="B24" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="C24" s="2">
+      <c r="C24" s="2" t="s">
+        <v>108</v>
+      </c>
+      <c r="D24" s="2">
         <v>4005</v>
       </c>
-      <c r="D24" s="2">
+      <c r="E24" s="2">
         <v>21.21</v>
       </c>
-      <c r="E24" s="2">
+      <c r="F24" s="2">
         <v>14882</v>
       </c>
-      <c r="F24" s="2">
+      <c r="G24" s="2">
         <v>14879</v>
       </c>
-      <c r="G24" s="2"/>
-      <c r="H24" s="18"/>
-      <c r="I24" s="18"/>
-    </row>
-    <row r="25" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="H24" s="2"/>
+    </row>
+    <row r="25" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A25" s="2" t="s">
         <v>14</v>
       </c>
       <c r="B25" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="C25" s="2">
+      <c r="C25" s="2" t="s">
+        <v>108</v>
+      </c>
+      <c r="D25" s="2">
         <v>1366</v>
       </c>
-      <c r="D25" s="2">
+      <c r="E25" s="2">
         <v>7.23</v>
       </c>
-      <c r="E25" s="2">
+      <c r="F25" s="2">
         <v>17521</v>
       </c>
-      <c r="F25" s="2">
+      <c r="G25" s="2">
         <v>17516</v>
       </c>
-      <c r="G25" s="2"/>
-      <c r="H25" s="18"/>
-      <c r="I25" s="18"/>
-      <c r="J25" s="5"/>
-    </row>
-    <row r="26" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="H25" s="2"/>
+      <c r="K25"/>
+    </row>
+    <row r="26" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A26" s="4" t="s">
         <v>28</v>
       </c>
       <c r="B26" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="C26" s="4">
+      <c r="C26" s="4" t="s">
+        <v>109</v>
+      </c>
+      <c r="D26" s="4">
         <v>1081</v>
       </c>
-      <c r="D26" s="4">
+      <c r="E26" s="4">
         <v>5.72</v>
       </c>
-      <c r="E26" s="4">
+      <c r="F26" s="4">
         <v>17806</v>
       </c>
-      <c r="F26" s="4">
+      <c r="G26" s="4">
         <v>9</v>
       </c>
-      <c r="G26" s="4"/>
-      <c r="H26" s="18"/>
-      <c r="I26" s="18"/>
-    </row>
-    <row r="27" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="H26" s="4"/>
+    </row>
+    <row r="27" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A27" s="2" t="s">
         <v>19</v>
       </c>
       <c r="B27" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="C27" s="2">
+      <c r="C27" s="2" t="s">
+        <v>108</v>
+      </c>
+      <c r="D27" s="2">
         <v>1011</v>
       </c>
-      <c r="D27" s="2">
+      <c r="E27" s="2">
         <v>5.35</v>
       </c>
-      <c r="E27" s="2">
+      <c r="F27" s="2">
         <v>17876</v>
       </c>
-      <c r="F27" s="2">
+      <c r="G27" s="2">
         <v>16044</v>
       </c>
-      <c r="G27" s="2"/>
-      <c r="H27" s="18" t="s">
+      <c r="H27" s="2"/>
+      <c r="I27" t="s">
         <v>43</v>
       </c>
-      <c r="I27" s="18" t="s">
+      <c r="J27" s="5" t="s">
         <v>76</v>
       </c>
     </row>
-    <row r="28" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A28" s="2" t="s">
         <v>18</v>
       </c>
       <c r="B28" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="C28" s="2">
+      <c r="C28" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="D28" s="2">
         <v>1011</v>
       </c>
-      <c r="D28" s="2">
+      <c r="E28" s="2">
         <v>5.35</v>
       </c>
-      <c r="E28" s="2">
+      <c r="F28" s="2">
         <v>17876</v>
       </c>
-      <c r="F28" s="2">
+      <c r="G28" s="2">
         <v>4359</v>
       </c>
-      <c r="G28" s="2"/>
-      <c r="H28" s="18"/>
-      <c r="I28" s="18"/>
-    </row>
-    <row r="29" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A29" s="11" t="s">
+      <c r="H28" s="2"/>
+    </row>
+    <row r="29" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A29" s="10" t="s">
         <v>77</v>
       </c>
-      <c r="B29" s="11" t="s">
-        <v>6</v>
-      </c>
-      <c r="C29" s="11">
+      <c r="B29" s="10" t="s">
+        <v>6</v>
+      </c>
+      <c r="C29" s="10" t="s">
+        <v>6</v>
+      </c>
+      <c r="D29" s="10">
         <v>931</v>
       </c>
-      <c r="D29" s="11">
+      <c r="E29" s="10">
         <v>4.93</v>
       </c>
-      <c r="E29" s="11">
+      <c r="F29" s="10">
         <v>17956</v>
       </c>
-      <c r="F29" s="11">
+      <c r="G29" s="10">
         <v>1214</v>
       </c>
-      <c r="G29" s="11"/>
-      <c r="H29" s="18"/>
-      <c r="I29" s="18"/>
-    </row>
-    <row r="30" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="H29" s="10"/>
+      <c r="K29" s="5" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="30" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A30" s="2" t="s">
         <v>10</v>
       </c>
       <c r="B30" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="C30" s="2">
+      <c r="C30" s="2" t="s">
+        <v>110</v>
+      </c>
+      <c r="D30" s="2">
         <v>921</v>
       </c>
-      <c r="D30" s="2">
+      <c r="E30" s="2">
         <v>4.88</v>
       </c>
-      <c r="E30" s="2">
+      <c r="F30" s="2">
         <v>17966</v>
       </c>
-      <c r="F30" s="2">
+      <c r="G30" s="2">
         <v>2</v>
       </c>
-      <c r="G30" s="2"/>
-      <c r="H30" s="18"/>
-      <c r="I30" s="18"/>
-    </row>
-    <row r="31" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="H30" s="2"/>
+    </row>
+    <row r="31" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A31" s="2" t="s">
         <v>12</v>
       </c>
       <c r="B31" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="C31" s="2">
+      <c r="C31" s="2" t="s">
+        <v>108</v>
+      </c>
+      <c r="D31" s="2">
         <v>646</v>
       </c>
-      <c r="D31" s="2">
+      <c r="E31" s="2">
         <v>3.42</v>
       </c>
-      <c r="E31" s="2">
+      <c r="F31" s="2">
         <v>18241</v>
       </c>
-      <c r="F31" s="2">
+      <c r="G31" s="2">
         <v>18050</v>
       </c>
-      <c r="G31" s="2"/>
-      <c r="H31" s="18"/>
-      <c r="I31" s="18"/>
-    </row>
-    <row r="32" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="H31" s="2"/>
+    </row>
+    <row r="32" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A32" s="1" t="s">
         <v>78</v>
       </c>
       <c r="B32" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="C32" s="1">
+      <c r="C32" s="1"/>
+      <c r="D32" s="1">
         <v>631</v>
       </c>
-      <c r="D32" s="1">
+      <c r="E32" s="1">
         <v>3.34</v>
       </c>
-      <c r="E32" s="1">
+      <c r="F32" s="1">
         <v>18256</v>
       </c>
-      <c r="F32" s="1">
+      <c r="G32" s="1">
         <v>1</v>
       </c>
-      <c r="G32" s="1"/>
-      <c r="H32" s="18"/>
-      <c r="I32" s="18" t="s">
+      <c r="H32" s="1"/>
+      <c r="J32" s="5" t="s">
         <v>57</v>
       </c>
     </row>
-    <row r="33" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A33" s="4" t="s">
         <v>36</v>
       </c>
       <c r="B33" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="C33" s="4">
+      <c r="C33" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="D33" s="4">
         <v>47</v>
       </c>
-      <c r="D33" s="4">
+      <c r="E33" s="4">
         <v>0.25</v>
       </c>
-      <c r="E33" s="4">
+      <c r="F33" s="4">
         <v>18840</v>
       </c>
-      <c r="F33" s="4">
+      <c r="G33" s="4">
         <v>5945</v>
       </c>
-      <c r="G33" s="4"/>
-      <c r="H33" s="18"/>
-      <c r="I33" s="18"/>
-    </row>
-    <row r="34" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="H33" s="4"/>
+    </row>
+    <row r="34" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A34" s="2" t="s">
         <v>27</v>
       </c>
       <c r="B34" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="C34" s="2">
+      <c r="C34" s="2" t="s">
+        <v>111</v>
+      </c>
+      <c r="D34" s="2">
         <v>27</v>
       </c>
-      <c r="D34" s="2">
+      <c r="E34" s="2">
         <v>0.14000000000000001</v>
       </c>
-      <c r="E34" s="2">
+      <c r="F34" s="2">
         <v>18860</v>
       </c>
-      <c r="F34" s="2">
+      <c r="G34" s="2">
         <v>30</v>
       </c>
-      <c r="G34" s="2"/>
-      <c r="H34" s="18"/>
-      <c r="I34" s="18"/>
-    </row>
-    <row r="35" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A35" s="12" t="s">
+      <c r="H34" s="2"/>
+    </row>
+    <row r="35" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A35" s="3" t="s">
         <v>30</v>
       </c>
-      <c r="B35" s="12" t="s">
-        <v>6</v>
-      </c>
-      <c r="C35" s="12">
+      <c r="B35" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="C35" s="3" t="s">
+        <v>109</v>
+      </c>
+      <c r="D35" s="3">
         <v>22</v>
       </c>
-      <c r="D35" s="12">
+      <c r="E35" s="3">
         <v>0.12</v>
       </c>
-      <c r="E35" s="12">
+      <c r="F35" s="3">
         <v>18865</v>
       </c>
-      <c r="F35" s="12">
+      <c r="G35" s="3">
         <v>4</v>
       </c>
-      <c r="G35" s="12"/>
-      <c r="H35" s="19"/>
-      <c r="I35" s="19"/>
-      <c r="J35" s="13"/>
-    </row>
-    <row r="36" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A36" s="12" t="s">
+      <c r="H35" s="3"/>
+    </row>
+    <row r="36" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A36" s="3" t="s">
         <v>24</v>
       </c>
-      <c r="B36" s="12" t="s">
-        <v>6</v>
-      </c>
-      <c r="C36" s="12">
+      <c r="B36" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="C36" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="D36" s="3">
         <v>22</v>
       </c>
-      <c r="D36" s="12">
+      <c r="E36" s="3">
         <v>0.12</v>
       </c>
-      <c r="E36" s="12">
+      <c r="F36" s="3">
         <v>18865</v>
       </c>
-      <c r="F36" s="12">
+      <c r="G36" s="3">
         <v>14512</v>
       </c>
-      <c r="G36" s="12"/>
-      <c r="H36" s="19" t="s">
+      <c r="H36" s="3"/>
+      <c r="I36" t="s">
         <v>79</v>
       </c>
-      <c r="I36" s="19" t="s">
+      <c r="J36" s="5" t="s">
         <v>80</v>
       </c>
-      <c r="J36" s="13"/>
-    </row>
-    <row r="37" spans="1:10" ht="16.8" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A37" s="14" t="s">
+      <c r="K36" s="5" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="37" spans="1:11" ht="16.8" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A37" s="1" t="s">
         <v>31</v>
       </c>
-      <c r="B37" s="14" t="s">
-        <v>6</v>
-      </c>
-      <c r="C37" s="14">
+      <c r="B37" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="C37" s="1"/>
+      <c r="D37" s="1">
         <v>21</v>
       </c>
-      <c r="D37" s="14">
+      <c r="E37" s="1">
         <v>0.11</v>
       </c>
-      <c r="E37" s="14">
+      <c r="F37" s="1">
         <v>18866</v>
       </c>
-      <c r="F37" s="14">
+      <c r="G37" s="1">
         <v>2</v>
       </c>
-      <c r="G37" s="14"/>
-      <c r="H37" s="19"/>
-      <c r="I37" s="19" t="s">
+      <c r="H37" s="1"/>
+      <c r="J37" s="5" t="s">
         <v>81</v>
       </c>
-      <c r="J37" s="13"/>
-    </row>
-    <row r="38" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A38" s="15" t="s">
+    </row>
+    <row r="38" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A38" s="4" t="s">
         <v>29</v>
       </c>
-      <c r="B38" s="15" t="s">
-        <v>6</v>
-      </c>
-      <c r="C38" s="15">
+      <c r="B38" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="C38" s="4" t="s">
+        <v>109</v>
+      </c>
+      <c r="D38" s="4">
         <v>15</v>
       </c>
-      <c r="D38" s="15">
+      <c r="E38" s="4">
         <v>0.08</v>
       </c>
-      <c r="E38" s="15">
+      <c r="F38" s="4">
         <v>18872</v>
       </c>
-      <c r="F38" s="15">
+      <c r="G38" s="4">
         <v>5</v>
       </c>
-      <c r="G38" s="15"/>
-      <c r="H38" s="19"/>
-      <c r="I38" s="19"/>
-      <c r="J38" s="16"/>
-    </row>
-    <row r="39" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A39" s="17" t="s">
+      <c r="H38" s="4"/>
+      <c r="K38"/>
+    </row>
+    <row r="39" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A39" s="2" t="s">
         <v>35</v>
       </c>
-      <c r="B39" s="17" t="s">
-        <v>6</v>
-      </c>
-      <c r="C39" s="17">
+      <c r="B39" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="C39" s="2" t="s">
+        <v>112</v>
+      </c>
+      <c r="D39" s="2">
         <v>5</v>
       </c>
-      <c r="D39" s="17">
+      <c r="E39" s="2">
         <v>0.03</v>
       </c>
-      <c r="E39" s="17">
+      <c r="F39" s="2">
         <v>18882</v>
       </c>
-      <c r="F39" s="17">
+      <c r="G39" s="2">
         <v>16323</v>
       </c>
-      <c r="G39" s="17"/>
-      <c r="H39" s="19"/>
-      <c r="I39" s="19"/>
-      <c r="J39" s="13"/>
-    </row>
-    <row r="40" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A40" s="17" t="s">
+      <c r="H39" s="2"/>
+    </row>
+    <row r="40" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A40" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="B40" s="17" t="s">
+      <c r="B40" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="C40" s="17">
-        <v>0</v>
-      </c>
-      <c r="D40" s="17">
-        <v>0</v>
-      </c>
-      <c r="E40" s="17">
+      <c r="C40" s="2" t="s">
+        <v>108</v>
+      </c>
+      <c r="D40" s="2">
+        <v>0</v>
+      </c>
+      <c r="E40" s="2">
+        <v>0</v>
+      </c>
+      <c r="F40" s="2">
         <v>18887</v>
       </c>
-      <c r="F40" s="17">
+      <c r="G40" s="2">
         <v>18540</v>
       </c>
-      <c r="G40" s="17"/>
-      <c r="H40" s="19"/>
-      <c r="I40" s="19"/>
-      <c r="J40" s="13"/>
-    </row>
-    <row r="41" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A41" s="17" t="s">
+      <c r="H40" s="2"/>
+    </row>
+    <row r="41" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A41" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="B41" s="17" t="s">
-        <v>6</v>
-      </c>
-      <c r="C41" s="17">
-        <v>0</v>
-      </c>
-      <c r="D41" s="17">
-        <v>0</v>
-      </c>
-      <c r="E41" s="17">
+      <c r="B41" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="C41" s="2" t="s">
+        <v>113</v>
+      </c>
+      <c r="D41" s="2">
+        <v>0</v>
+      </c>
+      <c r="E41" s="2">
+        <v>0</v>
+      </c>
+      <c r="F41" s="2">
         <v>18887</v>
       </c>
-      <c r="F41" s="17">
+      <c r="G41" s="2">
         <v>394</v>
       </c>
-      <c r="G41" s="17"/>
-      <c r="H41" s="19"/>
-      <c r="I41" s="19"/>
-      <c r="J41" s="13"/>
-    </row>
-    <row r="42" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A42" s="12" t="s">
+      <c r="H41" s="2"/>
+    </row>
+    <row r="42" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A42" s="3" t="s">
         <v>20</v>
       </c>
-      <c r="B42" s="12" t="s">
+      <c r="B42" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="C42" s="12">
-        <v>0</v>
-      </c>
-      <c r="D42" s="12">
-        <v>0</v>
-      </c>
-      <c r="E42" s="12">
+      <c r="C42" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="D42" s="3">
+        <v>0</v>
+      </c>
+      <c r="E42" s="3">
+        <v>0</v>
+      </c>
+      <c r="F42" s="3">
         <v>18887</v>
       </c>
-      <c r="F42" s="12">
+      <c r="G42" s="3">
         <v>7371</v>
       </c>
-      <c r="G42" s="12"/>
-      <c r="H42" s="19"/>
-      <c r="I42" s="19" t="s">
+      <c r="H42" s="3"/>
+      <c r="J42" s="5" t="s">
         <v>82</v>
       </c>
-      <c r="J42" s="13"/>
-    </row>
-    <row r="43" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A43" s="17" t="s">
+    </row>
+    <row r="43" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A43" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="B43" s="17" t="s">
-        <v>6</v>
-      </c>
-      <c r="C43" s="17">
-        <v>0</v>
-      </c>
-      <c r="D43" s="17">
-        <v>0</v>
-      </c>
-      <c r="E43" s="17">
+      <c r="B43" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="C43" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="D43" s="2">
+        <v>0</v>
+      </c>
+      <c r="E43" s="2">
+        <v>0</v>
+      </c>
+      <c r="F43" s="2">
         <v>18887</v>
       </c>
-      <c r="F43" s="17">
+      <c r="G43" s="2">
         <v>18887</v>
       </c>
-      <c r="G43" s="17"/>
-      <c r="H43" s="19"/>
-      <c r="I43" s="19"/>
-      <c r="J43" s="13"/>
-    </row>
-    <row r="44" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A44" s="3" t="s">
+      <c r="H43" s="2"/>
+    </row>
+    <row r="44" spans="1:11" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A44" s="12" t="s">
         <v>21</v>
       </c>
-      <c r="B44" s="3" t="s">
-        <v>6</v>
-      </c>
-      <c r="C44" s="3">
-        <v>0</v>
-      </c>
-      <c r="D44" s="3">
-        <v>0</v>
-      </c>
-      <c r="E44" s="3">
+      <c r="B44" s="12" t="s">
+        <v>6</v>
+      </c>
+      <c r="C44" s="12" t="s">
+        <v>6</v>
+      </c>
+      <c r="D44" s="12">
+        <v>0</v>
+      </c>
+      <c r="E44" s="12">
+        <v>0</v>
+      </c>
+      <c r="F44" s="12">
         <v>18887</v>
       </c>
-      <c r="F44" s="3">
+      <c r="G44" s="12">
         <v>32</v>
       </c>
-      <c r="G44" s="3"/>
-      <c r="H44" s="18"/>
-      <c r="I44" s="18"/>
-    </row>
-    <row r="61" ht="14.4" x14ac:dyDescent="0.3"/>
-    <row r="68" spans="10:10" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="J68" s="5"/>
+      <c r="H44" s="12"/>
+    </row>
+    <row r="45" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A45" s="10" t="s">
+        <v>88</v>
+      </c>
+      <c r="B45" s="10" t="s">
+        <v>89</v>
+      </c>
+      <c r="C45" s="10"/>
+      <c r="D45" s="10">
+        <v>0</v>
+      </c>
+      <c r="E45" s="10">
+        <v>0</v>
+      </c>
+      <c r="F45" s="10">
+        <v>17966</v>
+      </c>
+      <c r="G45" s="10">
+        <v>2</v>
+      </c>
+      <c r="H45" s="10"/>
+    </row>
+    <row r="46" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A46" s="3" t="s">
+        <v>90</v>
+      </c>
+      <c r="B46" s="3" t="s">
+        <v>89</v>
+      </c>
+      <c r="C46" s="3"/>
+      <c r="D46" s="3">
+        <v>0</v>
+      </c>
+      <c r="E46" s="3">
+        <v>0</v>
+      </c>
+      <c r="F46" s="3">
+        <v>17966</v>
+      </c>
+      <c r="G46" s="3">
+        <v>2</v>
+      </c>
+      <c r="H46" s="3"/>
+    </row>
+    <row r="47" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A47" s="2" t="s">
+        <v>91</v>
+      </c>
+      <c r="B47" s="2" t="s">
+        <v>89</v>
+      </c>
+      <c r="C47" s="2"/>
+      <c r="D47" s="2">
+        <v>0</v>
+      </c>
+      <c r="E47" s="2">
+        <v>0</v>
+      </c>
+      <c r="F47" s="2">
+        <v>17966</v>
+      </c>
+      <c r="G47" s="2">
+        <v>2</v>
+      </c>
+      <c r="H47" s="2"/>
+    </row>
+    <row r="48" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A48" s="10" t="s">
+        <v>92</v>
+      </c>
+      <c r="B48" s="10" t="s">
+        <v>89</v>
+      </c>
+      <c r="C48" s="10"/>
+      <c r="D48" s="10">
+        <v>0</v>
+      </c>
+      <c r="E48" s="10">
+        <v>0</v>
+      </c>
+      <c r="F48" s="10">
+        <v>17966</v>
+      </c>
+      <c r="G48" s="10">
+        <v>2</v>
+      </c>
+      <c r="H48" s="10"/>
+    </row>
+    <row r="49" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A49" s="10" t="s">
+        <v>93</v>
+      </c>
+      <c r="B49" s="10" t="s">
+        <v>11</v>
+      </c>
+      <c r="C49" s="10"/>
+      <c r="D49" s="10">
+        <v>1488</v>
+      </c>
+      <c r="E49" s="10">
+        <v>8.2799999999999994</v>
+      </c>
+      <c r="F49" s="10">
+        <v>16478</v>
+      </c>
+      <c r="G49" s="10">
+        <v>12</v>
+      </c>
+      <c r="H49" s="10"/>
+    </row>
+    <row r="50" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A50" t="s">
+        <v>94</v>
+      </c>
+      <c r="B50" t="s">
+        <v>89</v>
+      </c>
+      <c r="D50">
+        <v>0</v>
+      </c>
+      <c r="E50">
+        <v>0</v>
+      </c>
+      <c r="F50">
+        <v>17966</v>
+      </c>
+      <c r="G50">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="51" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A51" s="2" t="s">
+        <v>95</v>
+      </c>
+      <c r="B51" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="C51" s="2"/>
+      <c r="D51" s="2">
+        <v>0</v>
+      </c>
+      <c r="E51" s="2">
+        <v>0</v>
+      </c>
+      <c r="F51" s="2">
+        <v>17966</v>
+      </c>
+      <c r="G51" s="2">
+        <v>11</v>
+      </c>
+      <c r="H51" s="2"/>
+    </row>
+    <row r="52" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A52" t="s">
+        <v>96</v>
+      </c>
+      <c r="B52" t="s">
+        <v>89</v>
+      </c>
+      <c r="D52">
+        <v>0</v>
+      </c>
+      <c r="E52">
+        <v>0</v>
+      </c>
+      <c r="F52">
+        <v>17966</v>
+      </c>
+      <c r="G52">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="53" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A53" t="s">
+        <v>97</v>
+      </c>
+      <c r="B53" t="s">
+        <v>89</v>
+      </c>
+      <c r="D53">
+        <v>0</v>
+      </c>
+      <c r="E53">
+        <v>0</v>
+      </c>
+      <c r="F53">
+        <v>17966</v>
+      </c>
+      <c r="G53">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="54" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A54" t="s">
+        <v>98</v>
+      </c>
+      <c r="B54" t="s">
+        <v>89</v>
+      </c>
+      <c r="D54">
+        <v>0</v>
+      </c>
+      <c r="E54">
+        <v>0</v>
+      </c>
+      <c r="F54">
+        <v>17966</v>
+      </c>
+      <c r="G54">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="55" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A55" t="s">
+        <v>99</v>
+      </c>
+      <c r="B55" t="s">
+        <v>89</v>
+      </c>
+      <c r="D55">
+        <v>0</v>
+      </c>
+      <c r="E55">
+        <v>0</v>
+      </c>
+      <c r="F55">
+        <v>17966</v>
+      </c>
+      <c r="G55">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="56" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A56" t="s">
+        <v>100</v>
+      </c>
+      <c r="B56" t="s">
+        <v>89</v>
+      </c>
+      <c r="D56">
+        <v>0</v>
+      </c>
+      <c r="E56">
+        <v>0</v>
+      </c>
+      <c r="F56">
+        <v>17966</v>
+      </c>
+      <c r="G56">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="57" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A57" t="s">
+        <v>101</v>
+      </c>
+      <c r="B57" t="s">
+        <v>89</v>
+      </c>
+      <c r="D57">
+        <v>0</v>
+      </c>
+      <c r="E57">
+        <v>0</v>
+      </c>
+      <c r="F57">
+        <v>17966</v>
+      </c>
+      <c r="G57">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="58" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A58" t="s">
+        <v>102</v>
+      </c>
+      <c r="B58" t="s">
+        <v>89</v>
+      </c>
+      <c r="D58">
+        <v>0</v>
+      </c>
+      <c r="E58">
+        <v>0</v>
+      </c>
+      <c r="F58">
+        <v>17966</v>
+      </c>
+      <c r="G58">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="59" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A59" t="s">
+        <v>103</v>
+      </c>
+      <c r="B59" t="s">
+        <v>89</v>
+      </c>
+      <c r="D59">
+        <v>0</v>
+      </c>
+      <c r="E59">
+        <v>0</v>
+      </c>
+      <c r="F59">
+        <v>17966</v>
+      </c>
+      <c r="G59">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="60" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A60" t="s">
+        <v>104</v>
+      </c>
+      <c r="B60" t="s">
+        <v>89</v>
+      </c>
+      <c r="D60">
+        <v>0</v>
+      </c>
+      <c r="E60">
+        <v>0</v>
+      </c>
+      <c r="F60">
+        <v>17966</v>
+      </c>
+      <c r="G60">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="61" spans="1:8" ht="14.4" x14ac:dyDescent="0.3">
+      <c r="A61" t="s">
+        <v>105</v>
+      </c>
+      <c r="B61" t="s">
+        <v>89</v>
+      </c>
+      <c r="D61">
+        <v>0</v>
+      </c>
+      <c r="E61">
+        <v>0</v>
+      </c>
+      <c r="F61">
+        <v>17966</v>
+      </c>
+      <c r="G61">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="62" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A62" t="s">
+        <v>106</v>
+      </c>
+      <c r="B62" t="s">
+        <v>89</v>
+      </c>
+      <c r="D62">
+        <v>0</v>
+      </c>
+      <c r="E62">
+        <v>0</v>
+      </c>
+      <c r="F62">
+        <v>17966</v>
+      </c>
+      <c r="G62">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="63" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A63" t="s">
+        <v>114</v>
+      </c>
+      <c r="B63" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="64" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A64" t="s">
+        <v>115</v>
+      </c>
+      <c r="B64" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="65" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A65" t="s">
+        <v>116</v>
+      </c>
+      <c r="B65" t="s">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="66" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A66" t="s">
+        <v>117</v>
+      </c>
+      <c r="B66" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="68" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="K68"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:I1" xr:uid="{00000000-0001-0000-0000-000000000000}"/>
+  <autoFilter ref="A1:J1" xr:uid="{00000000-0001-0000-0000-000000000000}"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup paperSize="9" orientation="landscape" r:id="rId1"/>
 </worksheet>

</xml_diff>